<commit_message>
Studio 9: link the Smartsheet workbook and notebook; reconcile AI against the notebook
The header lists all three files. Part 5 now has students enter Gemini's
two-coordinator schedule beside the notebook's optimum, run the three
feasibility checks on it, say which of their three schedules it matches,
and test its claim of optimality. The workbook's Reconciliation sheet
gains the matching columns and rows.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/week-09-resource-studio.xlsx
+++ b/files/week-09-resource-studio.xlsx
@@ -11756,13 +11756,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
@@ -11770,14 +11770,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI levelling · reconciliation</t>
+          <t>AI against the notebook · reconciliation</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gemini levels the two-coordinator case cold. Compare its schedule with yours and with the optimum, line by line.</t>
+          <t>Gemini levels the two-coordinator case cold. Enter its values beside the Colab notebook's optimum, line by line; the notebook is the reference.</t>
         </is>
       </c>
     </row>
@@ -11789,7 +11789,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Your value</t>
+          <t>Your value (Part 2)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -11799,7 +11799,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Optimum</t>
+          <t>Notebook optimum</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -11912,7 +11912,7 @@
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>Where it put the five-day loan</t>
+          <t>Claims shortest possible? True?</t>
         </is>
       </c>
       <c r="B13" s="15" t="n"/>
@@ -11924,7 +11924,7 @@
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Which of the three does it match?</t>
         </is>
       </c>
       <c r="B14" s="15" t="n"/>
@@ -11933,6 +11933,18 @@
       <c r="E14" s="15" t="n"/>
       <c r="F14" s="15" t="n"/>
     </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n"/>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="15" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish site (gated as of build date) 8f07acad5538864acb19956be4fcc62857484e94
</commit_message>
<xml_diff>
--- a/files/week-09-resource-studio.xlsx
+++ b/files/week-09-resource-studio.xlsx
@@ -11756,13 +11756,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
@@ -11770,14 +11770,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI levelling · reconciliation</t>
+          <t>AI against the notebook · reconciliation</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gemini levels the two-coordinator case cold. Compare its schedule with yours and with the optimum, line by line.</t>
+          <t>Gemini levels the two-coordinator case cold. Enter its values beside the Colab notebook's optimum, line by line; the notebook is the reference.</t>
         </is>
       </c>
     </row>
@@ -11789,7 +11789,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Your value</t>
+          <t>Your value (Part 2)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -11799,7 +11799,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Optimum</t>
+          <t>Notebook optimum</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -11912,7 +11912,7 @@
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>Where it put the five-day loan</t>
+          <t>Claims shortest possible? True?</t>
         </is>
       </c>
       <c r="B13" s="15" t="n"/>
@@ -11924,7 +11924,7 @@
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Which of the three does it match?</t>
         </is>
       </c>
       <c r="B14" s="15" t="n"/>
@@ -11933,6 +11933,18 @@
       <c r="E14" s="15" t="n"/>
       <c r="F14" s="15" t="n"/>
     </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n"/>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="15" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>